<commit_message>
fix(template): populate precalculated total attendance values in summary rows
</commit_message>
<xml_diff>
--- a/assets/templates/Adidata_master_template.xlsx
+++ b/assets/templates/Adidata_master_template.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\901810\GitHub\timesheet-generator\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885D1BE1-6FB5-4309-8625-4A850FEA2DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="SPL_TEMPLATE" sheetId="2" r:id="rId10"/>
+    <sheet name="SPL_TEMPLATE" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="53">
   <si>
     <t>NAME of PROJECT</t>
   </si>
@@ -198,130 +199,127 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <numFmts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-mmm\-yy"/>
-    <numFmt numFmtId="165" formatCode="d-mmm-yy"/>
-    <numFmt numFmtId="166" formatCode="h:mm"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <color rgb="FF000000"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="10"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Verdana"/>
-      <color rgb="FF000000"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
       <name val="Verdana"/>
-      <color rgb="FF333333"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Verdana"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="8"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <color theme="1"/>
-      <sz val="8"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color/>
-      <sz val="10"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color/>
-      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -348,23 +346,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF999999"/>
-        <bgColor rgb="FF999999"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFAEAAAA"/>
       </patternFill>
     </fill>
   </fills>
@@ -576,325 +558,296 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="20" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="16" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="20" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="17" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="17" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="4" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="true" applyBorder="true" applyAlignment="false">
-      <alignment/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="18" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="false">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -946,7 +899,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
@@ -962,9 +915,15 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="false"/>
+          <a:picLocks/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -978,16 +937,18 @@
           <a:off x="0" y="0"/>
           <a:ext cx="1285875" cy="238125"/>
         </a:xfrm>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+    <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1215,10 +1176,10 @@
       <c r="R1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="24.75" customHeight="1">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="63"/>
+      <c r="C2" s="62"/>
       <c r="D2" s="3" t="s">
         <v>33</v>
       </c>
@@ -1237,15 +1198,15 @@
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="18.75" customHeight="1">
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="64" t="s">
+      <c r="C3" s="62"/>
+      <c r="D3" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="4"/>
@@ -1263,10 +1224,10 @@
         <v>2</v>
       </c>
       <c r="C4" s="8"/>
-      <c r="D4" s="64" t="s">
+      <c r="D4" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="63"/>
+      <c r="E4" s="62"/>
       <c r="F4" s="9"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
@@ -1281,16 +1242,16 @@
       <c r="R4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="17.25" customHeight="1">
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="63"/>
-      <c r="D5" s="64" t="s">
+      <c r="C5" s="62"/>
+      <c r="D5" s="84" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
       <c r="H5" s="7"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -1303,10 +1264,10 @@
       <c r="R5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="17.25" customHeight="1">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="63"/>
+      <c r="C6" s="62"/>
       <c r="D6" s="10" t="s">
         <v>33</v>
       </c>
@@ -1314,18 +1275,18 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="11"/>
-      <c r="I6" s="65" t="s">
+      <c r="I6" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="J6" s="63"/>
+      <c r="J6" s="62"/>
       <c r="N6" s="1"/>
       <c r="O6" s="4"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="17.25" customHeight="1">
-      <c r="D7" s="66"/>
-      <c r="E7" s="67"/>
+      <c r="D7" s="79"/>
+      <c r="E7" s="65"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
       <c r="H7" s="13" t="s">
@@ -1350,51 +1311,51 @@
       <c r="Z7" s="16"/>
     </row>
     <row r="8" spans="1:26" ht="17.25" customHeight="1">
-      <c r="B8" s="68" t="s">
+      <c r="B8" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="70" t="s">
+      <c r="C8" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="71"/>
-      <c r="E8" s="72" t="s">
+      <c r="D8" s="57"/>
+      <c r="E8" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="73" t="s">
+      <c r="F8" s="83" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="74"/>
-      <c r="J8" s="74"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="75" t="s">
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
+      <c r="J8" s="56"/>
+      <c r="K8" s="57"/>
+      <c r="L8" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="M8" s="76"/>
-      <c r="N8" s="77"/>
-      <c r="O8" s="94" t="s">
+      <c r="M8" s="59"/>
+      <c r="N8" s="60"/>
+      <c r="O8" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="P8" s="94" t="s">
+      <c r="P8" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="Q8" s="95" t="s">
+      <c r="Q8" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="R8" s="95" t="s">
+      <c r="R8" s="54" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="23.25" customHeight="1">
-      <c r="B9" s="69"/>
+      <c r="B9" s="53"/>
       <c r="C9" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="69"/>
+      <c r="E9" s="53"/>
       <c r="F9" s="19" t="s">
         <v>18</v>
       </c>
@@ -1413,18 +1374,18 @@
       <c r="K9" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="L9" s="78"/>
-      <c r="M9" s="67"/>
-      <c r="N9" s="79"/>
-      <c r="O9" s="69"/>
-      <c r="P9" s="69"/>
-      <c r="Q9" s="69"/>
-      <c r="R9" s="69"/>
+      <c r="L9" s="64"/>
+      <c r="M9" s="65"/>
+      <c r="N9" s="66"/>
+      <c r="O9" s="53"/>
+      <c r="P9" s="53"/>
+      <c r="Q9" s="53"/>
+      <c r="R9" s="53"/>
     </row>
     <row r="10" spans="1:26" ht="15" customHeight="1">
       <c r="A10" s="20"/>
       <c r="B10" s="21">
-        <v>45383</v>
+        <v>45474</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>24</v>
@@ -1441,9 +1402,9 @@
       <c r="I10" s="23"/>
       <c r="J10" s="23"/>
       <c r="K10" s="24"/>
-      <c r="L10" s="80"/>
-      <c r="M10" s="74"/>
-      <c r="N10" s="71"/>
+      <c r="L10" s="74"/>
+      <c r="M10" s="56"/>
+      <c r="N10" s="57"/>
       <c r="O10" s="25"/>
       <c r="P10" s="25"/>
       <c r="Q10" s="25"/>
@@ -1459,20 +1420,26 @@
     </row>
     <row r="11" spans="1:26" ht="15" customHeight="1">
       <c r="B11" s="21">
-        <v>45384</v>
-      </c>
-      <c r="C11" s="22"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
+        <v>45475</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F11" s="23"/>
       <c r="G11" s="23"/>
       <c r="H11" s="23"/>
       <c r="I11" s="23"/>
       <c r="J11" s="23"/>
       <c r="K11" s="27"/>
-      <c r="L11" s="81"/>
-      <c r="M11" s="74"/>
-      <c r="N11" s="71"/>
+      <c r="L11" s="75"/>
+      <c r="M11" s="56"/>
+      <c r="N11" s="57"/>
       <c r="O11" s="28"/>
       <c r="P11" s="28"/>
       <c r="Q11" s="26"/>
@@ -1480,11 +1447,17 @@
     </row>
     <row r="12" spans="1:26" ht="15" customHeight="1">
       <c r="B12" s="21">
-        <v>45385</v>
-      </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
+        <v>45476</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F12" s="23"/>
       <c r="G12" s="23"/>
       <c r="H12" s="23"/>
@@ -1501,11 +1474,17 @@
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
       <c r="B13" s="21">
-        <v>45386</v>
-      </c>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
+        <v>45477</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F13" s="23"/>
       <c r="G13" s="23"/>
       <c r="H13" s="23"/>
@@ -1522,20 +1501,26 @@
     </row>
     <row r="14" spans="1:26" ht="15" customHeight="1">
       <c r="B14" s="21">
-        <v>45387</v>
-      </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
+        <v>45478</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F14" s="23"/>
       <c r="G14" s="23"/>
       <c r="H14" s="23"/>
       <c r="I14" s="23"/>
       <c r="J14" s="33"/>
       <c r="K14" s="27"/>
-      <c r="L14" s="82"/>
-      <c r="M14" s="74"/>
-      <c r="N14" s="71"/>
+      <c r="L14" s="76"/>
+      <c r="M14" s="56"/>
+      <c r="N14" s="57"/>
       <c r="O14" s="25"/>
       <c r="P14" s="25"/>
       <c r="Q14" s="31"/>
@@ -1543,11 +1528,17 @@
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1">
       <c r="B15" s="21">
-        <v>45388</v>
-      </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
+        <v>45479</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
       <c r="H15" s="35"/>
@@ -1564,11 +1555,17 @@
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1">
       <c r="B16" s="21">
-        <v>45389</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+        <v>45480</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="F16" s="23"/>
       <c r="G16" s="23"/>
       <c r="H16" s="23"/>
@@ -1585,674 +1582,820 @@
     </row>
     <row r="17" spans="2:18" ht="15" customHeight="1">
       <c r="B17" s="21">
-        <v>45390</v>
-      </c>
-      <c r="C17" s="43"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="44"/>
-      <c r="J17" s="44"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="83"/>
-      <c r="M17" s="74"/>
-      <c r="N17" s="71"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="46"/>
-      <c r="Q17" s="47"/>
-      <c r="R17" s="48"/>
+        <v>45481</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
+      <c r="K17" s="90"/>
+      <c r="L17" s="91"/>
+      <c r="M17" s="92"/>
+      <c r="N17" s="93"/>
+      <c r="O17" s="94"/>
+      <c r="P17" s="94"/>
+      <c r="Q17" s="95"/>
+      <c r="R17" s="96"/>
     </row>
     <row r="18" spans="2:18" ht="15" customHeight="1">
       <c r="B18" s="21">
-        <v>45391</v>
-      </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="44"/>
-      <c r="J18" s="44"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="83"/>
-      <c r="M18" s="74"/>
-      <c r="N18" s="71"/>
-      <c r="O18" s="46"/>
-      <c r="P18" s="46"/>
-      <c r="Q18" s="47"/>
-      <c r="R18" s="48"/>
+        <v>45482</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18" s="89"/>
+      <c r="G18" s="89"/>
+      <c r="H18" s="89"/>
+      <c r="I18" s="89"/>
+      <c r="J18" s="89"/>
+      <c r="K18" s="97"/>
+      <c r="L18" s="91"/>
+      <c r="M18" s="92"/>
+      <c r="N18" s="93"/>
+      <c r="O18" s="94"/>
+      <c r="P18" s="94"/>
+      <c r="Q18" s="95"/>
+      <c r="R18" s="96"/>
     </row>
     <row r="19" spans="2:18" ht="14.4">
       <c r="B19" s="21">
-        <v>45392</v>
-      </c>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="44"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="83"/>
-      <c r="M19" s="74"/>
-      <c r="N19" s="71"/>
-      <c r="O19" s="46"/>
-      <c r="P19" s="46"/>
-      <c r="Q19" s="47"/>
-      <c r="R19" s="48"/>
+        <v>45483</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="89"/>
+      <c r="G19" s="89"/>
+      <c r="H19" s="89"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="89"/>
+      <c r="K19" s="97"/>
+      <c r="L19" s="91"/>
+      <c r="M19" s="92"/>
+      <c r="N19" s="93"/>
+      <c r="O19" s="94"/>
+      <c r="P19" s="94"/>
+      <c r="Q19" s="95"/>
+      <c r="R19" s="96"/>
     </row>
     <row r="20" spans="2:18" ht="14.4">
       <c r="B20" s="21">
-        <v>45393</v>
-      </c>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="44"/>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="83"/>
-      <c r="M20" s="74"/>
-      <c r="N20" s="71"/>
-      <c r="O20" s="46"/>
-      <c r="P20" s="46"/>
-      <c r="Q20" s="47"/>
-      <c r="R20" s="48"/>
+        <v>45484</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="89"/>
+      <c r="G20" s="89"/>
+      <c r="H20" s="89"/>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="97"/>
+      <c r="L20" s="91"/>
+      <c r="M20" s="92"/>
+      <c r="N20" s="93"/>
+      <c r="O20" s="94"/>
+      <c r="P20" s="94"/>
+      <c r="Q20" s="95"/>
+      <c r="R20" s="96"/>
     </row>
     <row r="21" spans="2:18" ht="14.4">
       <c r="B21" s="21">
-        <v>45394</v>
-      </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="44"/>
-      <c r="H21" s="44"/>
-      <c r="I21" s="44"/>
-      <c r="J21" s="44"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="83"/>
-      <c r="M21" s="74"/>
-      <c r="N21" s="71"/>
-      <c r="O21" s="46"/>
-      <c r="P21" s="46"/>
-      <c r="Q21" s="47"/>
-      <c r="R21" s="48"/>
+        <v>45485</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21" s="89"/>
+      <c r="G21" s="89"/>
+      <c r="H21" s="89"/>
+      <c r="I21" s="89"/>
+      <c r="J21" s="89"/>
+      <c r="K21" s="97"/>
+      <c r="L21" s="91"/>
+      <c r="M21" s="92"/>
+      <c r="N21" s="93"/>
+      <c r="O21" s="94"/>
+      <c r="P21" s="94"/>
+      <c r="Q21" s="95"/>
+      <c r="R21" s="96"/>
     </row>
     <row r="22" spans="2:18" ht="14.4">
       <c r="B22" s="21">
-        <v>45395</v>
-      </c>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="44"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="44"/>
-      <c r="J22" s="44"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="83"/>
-      <c r="M22" s="74"/>
-      <c r="N22" s="71"/>
-      <c r="O22" s="46"/>
-      <c r="P22" s="46"/>
-      <c r="Q22" s="47"/>
-      <c r="R22" s="48"/>
+        <v>45486</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="89"/>
+      <c r="G22" s="89"/>
+      <c r="H22" s="89"/>
+      <c r="I22" s="89"/>
+      <c r="J22" s="89"/>
+      <c r="K22" s="97"/>
+      <c r="L22" s="91"/>
+      <c r="M22" s="92"/>
+      <c r="N22" s="93"/>
+      <c r="O22" s="94"/>
+      <c r="P22" s="94"/>
+      <c r="Q22" s="95"/>
+      <c r="R22" s="96"/>
     </row>
     <row r="23" spans="2:18" ht="14.4">
       <c r="B23" s="21">
-        <v>45396</v>
-      </c>
-      <c r="C23" s="43"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="44"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="83"/>
-      <c r="M23" s="74"/>
-      <c r="N23" s="71"/>
-      <c r="O23" s="46"/>
-      <c r="P23" s="46"/>
-      <c r="Q23" s="47"/>
-      <c r="R23" s="48"/>
+        <v>45487</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="89"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="89"/>
+      <c r="I23" s="89"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="97"/>
+      <c r="L23" s="91"/>
+      <c r="M23" s="92"/>
+      <c r="N23" s="93"/>
+      <c r="O23" s="94"/>
+      <c r="P23" s="94"/>
+      <c r="Q23" s="95"/>
+      <c r="R23" s="96"/>
     </row>
     <row r="24" spans="2:18" ht="14.4">
       <c r="B24" s="21">
-        <v>45397</v>
-      </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-      <c r="I24" s="44"/>
-      <c r="J24" s="44"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="83"/>
-      <c r="M24" s="74"/>
-      <c r="N24" s="71"/>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
-      <c r="Q24" s="47"/>
-      <c r="R24" s="48"/>
+        <v>45488</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="89"/>
+      <c r="G24" s="89"/>
+      <c r="H24" s="89"/>
+      <c r="I24" s="89"/>
+      <c r="J24" s="89"/>
+      <c r="K24" s="97"/>
+      <c r="L24" s="91"/>
+      <c r="M24" s="92"/>
+      <c r="N24" s="93"/>
+      <c r="O24" s="94"/>
+      <c r="P24" s="94"/>
+      <c r="Q24" s="95"/>
+      <c r="R24" s="96"/>
     </row>
     <row r="25" spans="2:18" ht="14.4">
       <c r="B25" s="21">
-        <v>45398</v>
-      </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="27"/>
-      <c r="L25" s="29"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="25"/>
-      <c r="P25" s="25"/>
-      <c r="Q25" s="31"/>
-      <c r="R25" s="26"/>
+        <v>45489</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25" s="89"/>
+      <c r="G25" s="89"/>
+      <c r="H25" s="89"/>
+      <c r="I25" s="89"/>
+      <c r="J25" s="89"/>
+      <c r="K25" s="97"/>
+      <c r="L25" s="98"/>
+      <c r="M25" s="98"/>
+      <c r="N25" s="99"/>
+      <c r="O25" s="94"/>
+      <c r="P25" s="94"/>
+      <c r="Q25" s="95"/>
+      <c r="R25" s="96"/>
     </row>
     <row r="26" spans="2:18" ht="14.4">
       <c r="B26" s="21">
-        <v>45399</v>
-      </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="25"/>
-      <c r="P26" s="25"/>
-      <c r="Q26" s="31"/>
-      <c r="R26" s="26"/>
+        <v>45490</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26" s="89"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
+      <c r="I26" s="89"/>
+      <c r="J26" s="89"/>
+      <c r="K26" s="97"/>
+      <c r="L26" s="98"/>
+      <c r="M26" s="98"/>
+      <c r="N26" s="99"/>
+      <c r="O26" s="94"/>
+      <c r="P26" s="94"/>
+      <c r="Q26" s="95"/>
+      <c r="R26" s="96"/>
     </row>
     <row r="27" spans="2:18" ht="15" customHeight="1">
       <c r="B27" s="21">
-        <v>45400</v>
-      </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="29"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="25"/>
-      <c r="P27" s="25"/>
-      <c r="Q27" s="31"/>
-      <c r="R27" s="26"/>
+        <v>45491</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F27" s="89"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="89"/>
+      <c r="I27" s="89"/>
+      <c r="J27" s="89"/>
+      <c r="K27" s="97"/>
+      <c r="L27" s="98"/>
+      <c r="M27" s="98"/>
+      <c r="N27" s="99"/>
+      <c r="O27" s="94"/>
+      <c r="P27" s="94"/>
+      <c r="Q27" s="95"/>
+      <c r="R27" s="96"/>
     </row>
     <row r="28" spans="2:18" ht="14.4">
       <c r="B28" s="21">
-        <v>45401</v>
-      </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="25"/>
-      <c r="P28" s="25"/>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="26"/>
+        <v>45492</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" s="89"/>
+      <c r="G28" s="89"/>
+      <c r="H28" s="89"/>
+      <c r="I28" s="89"/>
+      <c r="J28" s="89"/>
+      <c r="K28" s="97"/>
+      <c r="L28" s="98"/>
+      <c r="M28" s="98"/>
+      <c r="N28" s="99"/>
+      <c r="O28" s="94"/>
+      <c r="P28" s="94"/>
+      <c r="Q28" s="95"/>
+      <c r="R28" s="96"/>
     </row>
     <row r="29" spans="2:18" ht="14.4">
       <c r="B29" s="21">
-        <v>45402</v>
-      </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="29"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="25"/>
-      <c r="P29" s="25"/>
-      <c r="Q29" s="31"/>
-      <c r="R29" s="26"/>
+        <v>45493</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="89"/>
+      <c r="G29" s="89"/>
+      <c r="H29" s="89"/>
+      <c r="I29" s="89"/>
+      <c r="J29" s="89"/>
+      <c r="K29" s="97"/>
+      <c r="L29" s="98"/>
+      <c r="M29" s="98"/>
+      <c r="N29" s="99"/>
+      <c r="O29" s="94"/>
+      <c r="P29" s="94"/>
+      <c r="Q29" s="95"/>
+      <c r="R29" s="96"/>
     </row>
     <row r="30" spans="2:18" ht="13.5" customHeight="1">
       <c r="B30" s="21">
-        <v>45403</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="29"/>
-      <c r="M30" s="29"/>
-      <c r="N30" s="30"/>
-      <c r="O30" s="25"/>
-      <c r="P30" s="25"/>
-      <c r="Q30" s="31"/>
-      <c r="R30" s="26"/>
+        <v>45494</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="89"/>
+      <c r="G30" s="89"/>
+      <c r="H30" s="89"/>
+      <c r="I30" s="89"/>
+      <c r="J30" s="89"/>
+      <c r="K30" s="97"/>
+      <c r="L30" s="98"/>
+      <c r="M30" s="98"/>
+      <c r="N30" s="99"/>
+      <c r="O30" s="94"/>
+      <c r="P30" s="94"/>
+      <c r="Q30" s="95"/>
+      <c r="R30" s="96"/>
     </row>
     <row r="31" spans="2:18" ht="14.4">
       <c r="B31" s="21">
-        <v>45404</v>
-      </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="29"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="30"/>
-      <c r="O31" s="25"/>
-      <c r="P31" s="25"/>
-      <c r="Q31" s="31"/>
-      <c r="R31" s="26"/>
+        <v>45495</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" s="89"/>
+      <c r="G31" s="89"/>
+      <c r="H31" s="89"/>
+      <c r="I31" s="89"/>
+      <c r="J31" s="89"/>
+      <c r="K31" s="97"/>
+      <c r="L31" s="98"/>
+      <c r="M31" s="98"/>
+      <c r="N31" s="99"/>
+      <c r="O31" s="94"/>
+      <c r="P31" s="94"/>
+      <c r="Q31" s="95"/>
+      <c r="R31" s="96"/>
     </row>
     <row r="32" spans="2:18" ht="14.4">
       <c r="B32" s="21">
-        <v>45405</v>
-      </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="29"/>
-      <c r="M32" s="29"/>
-      <c r="N32" s="30"/>
-      <c r="O32" s="25"/>
-      <c r="P32" s="25"/>
-      <c r="Q32" s="31"/>
-      <c r="R32" s="26"/>
+        <v>45496</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" s="89"/>
+      <c r="G32" s="89"/>
+      <c r="H32" s="89"/>
+      <c r="I32" s="89"/>
+      <c r="J32" s="89"/>
+      <c r="K32" s="97"/>
+      <c r="L32" s="98"/>
+      <c r="M32" s="98"/>
+      <c r="N32" s="99"/>
+      <c r="O32" s="94"/>
+      <c r="P32" s="94"/>
+      <c r="Q32" s="95"/>
+      <c r="R32" s="96"/>
     </row>
     <row r="33" spans="1:26" ht="14.4">
       <c r="B33" s="21">
-        <v>45406</v>
-      </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="23"/>
-      <c r="K33" s="27"/>
-      <c r="L33" s="29"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="30"/>
-      <c r="O33" s="25"/>
-      <c r="P33" s="25"/>
-      <c r="Q33" s="31"/>
-      <c r="R33" s="26"/>
+        <v>45497</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D33" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F33" s="89"/>
+      <c r="G33" s="89"/>
+      <c r="H33" s="89"/>
+      <c r="I33" s="89"/>
+      <c r="J33" s="89"/>
+      <c r="K33" s="97"/>
+      <c r="L33" s="98"/>
+      <c r="M33" s="98"/>
+      <c r="N33" s="99"/>
+      <c r="O33" s="94"/>
+      <c r="P33" s="94"/>
+      <c r="Q33" s="95"/>
+      <c r="R33" s="96"/>
     </row>
     <row r="34" spans="1:26" ht="14.4">
       <c r="B34" s="21">
-        <v>45407</v>
-      </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="27"/>
-      <c r="L34" s="29"/>
-      <c r="M34" s="29"/>
-      <c r="N34" s="30"/>
-      <c r="O34" s="25"/>
-      <c r="P34" s="25"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="26"/>
+        <v>45498</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" s="89"/>
+      <c r="G34" s="89"/>
+      <c r="H34" s="89"/>
+      <c r="I34" s="89"/>
+      <c r="J34" s="89"/>
+      <c r="K34" s="97"/>
+      <c r="L34" s="98"/>
+      <c r="M34" s="98"/>
+      <c r="N34" s="99"/>
+      <c r="O34" s="94"/>
+      <c r="P34" s="94"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="96"/>
     </row>
     <row r="35" spans="1:26" ht="14.4">
       <c r="B35" s="21">
-        <v>45408</v>
-      </c>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="50"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="29"/>
-      <c r="M35" s="29"/>
-      <c r="N35" s="30"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="25"/>
-      <c r="Q35" s="31"/>
-      <c r="R35" s="26"/>
+        <v>45499</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" s="100"/>
+      <c r="G35" s="100"/>
+      <c r="H35" s="100"/>
+      <c r="I35" s="100"/>
+      <c r="J35" s="100"/>
+      <c r="K35" s="97"/>
+      <c r="L35" s="98"/>
+      <c r="M35" s="98"/>
+      <c r="N35" s="99"/>
+      <c r="O35" s="94"/>
+      <c r="P35" s="94"/>
+      <c r="Q35" s="95"/>
+      <c r="R35" s="96"/>
     </row>
     <row r="36" spans="1:26" ht="14.4">
       <c r="B36" s="21">
-        <v>45409</v>
-      </c>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="29"/>
-      <c r="M36" s="29"/>
-      <c r="N36" s="51"/>
-      <c r="O36" s="25"/>
-      <c r="P36" s="25"/>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="26"/>
+        <v>45500</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" s="89"/>
+      <c r="G36" s="89"/>
+      <c r="H36" s="89"/>
+      <c r="I36" s="89"/>
+      <c r="J36" s="89"/>
+      <c r="K36" s="97"/>
+      <c r="L36" s="98"/>
+      <c r="M36" s="98"/>
+      <c r="N36" s="101"/>
+      <c r="O36" s="94"/>
+      <c r="P36" s="94"/>
+      <c r="Q36" s="95"/>
+      <c r="R36" s="96"/>
     </row>
     <row r="37" spans="1:26" ht="14.4">
       <c r="B37" s="21">
-        <v>45410</v>
-      </c>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="23"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="N37" s="52"/>
-      <c r="O37" s="25"/>
-      <c r="P37" s="25"/>
-      <c r="Q37" s="31"/>
-      <c r="R37" s="26"/>
+        <v>45501</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D37" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F37" s="89"/>
+      <c r="G37" s="89"/>
+      <c r="H37" s="89"/>
+      <c r="I37" s="89"/>
+      <c r="J37" s="89"/>
+      <c r="K37" s="97"/>
+      <c r="L37" s="98"/>
+      <c r="M37" s="98"/>
+      <c r="N37" s="102"/>
+      <c r="O37" s="94"/>
+      <c r="P37" s="94"/>
+      <c r="Q37" s="95"/>
+      <c r="R37" s="96"/>
     </row>
     <row r="38" spans="1:26" ht="15" customHeight="1">
       <c r="B38" s="21">
-        <v>45411</v>
-      </c>
-      <c r="C38" s="53"/>
-      <c r="D38" s="53"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23"/>
-      <c r="H38" s="23"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="23"/>
-      <c r="K38" s="27"/>
-      <c r="L38" s="29"/>
-      <c r="M38" s="29"/>
-      <c r="N38" s="54"/>
-      <c r="O38" s="25"/>
-      <c r="P38" s="25"/>
-      <c r="Q38" s="31"/>
-      <c r="R38" s="26"/>
+        <v>45502</v>
+      </c>
+      <c r="C38" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" s="89"/>
+      <c r="G38" s="89"/>
+      <c r="H38" s="89"/>
+      <c r="I38" s="89"/>
+      <c r="J38" s="89"/>
+      <c r="K38" s="97"/>
+      <c r="L38" s="98"/>
+      <c r="M38" s="98"/>
+      <c r="N38" s="103"/>
+      <c r="O38" s="94"/>
+      <c r="P38" s="94"/>
+      <c r="Q38" s="95"/>
+      <c r="R38" s="96"/>
     </row>
     <row r="39" spans="1:26" ht="15" customHeight="1">
       <c r="B39" s="21">
-        <v>45412</v>
-      </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="23"/>
-      <c r="K39" s="27"/>
-      <c r="L39" s="29"/>
-      <c r="M39" s="29"/>
-      <c r="N39" s="54"/>
-      <c r="O39" s="25"/>
-      <c r="P39" s="25"/>
-      <c r="Q39" s="31"/>
-      <c r="R39" s="26"/>
+        <v>45503</v>
+      </c>
+      <c r="C39" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E39" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F39" s="89"/>
+      <c r="G39" s="89"/>
+      <c r="H39" s="89"/>
+      <c r="I39" s="89"/>
+      <c r="J39" s="89"/>
+      <c r="K39" s="97"/>
+      <c r="L39" s="98"/>
+      <c r="M39" s="98"/>
+      <c r="N39" s="103"/>
+      <c r="O39" s="94"/>
+      <c r="P39" s="94"/>
+      <c r="Q39" s="95"/>
+      <c r="R39" s="96"/>
     </row>
     <row r="40" spans="1:26" ht="15" customHeight="1">
-      <c r="B40" s="21"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="43"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="44"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="49"/>
-      <c r="L40" s="55"/>
-      <c r="M40" s="55"/>
-      <c r="N40" s="56"/>
-      <c r="O40" s="57"/>
-      <c r="P40" s="57"/>
-      <c r="Q40" s="47"/>
-      <c r="R40" s="48"/>
+      <c r="B40" s="21">
+        <v>45504</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D40" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E40" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="89"/>
+      <c r="G40" s="89"/>
+      <c r="H40" s="89"/>
+      <c r="I40" s="89"/>
+      <c r="J40" s="89"/>
+      <c r="K40" s="97"/>
+      <c r="L40" s="104"/>
+      <c r="M40" s="104"/>
+      <c r="N40" s="105"/>
+      <c r="O40" s="106"/>
+      <c r="P40" s="106"/>
+      <c r="Q40" s="95"/>
+      <c r="R40" s="96"/>
     </row>
     <row r="41" spans="1:26" ht="15" customHeight="1">
-      <c r="B41" s="84"/>
-      <c r="C41" s="74"/>
-      <c r="D41" s="74"/>
-      <c r="E41" s="71"/>
-      <c r="F41" s="58">
+      <c r="B41" s="70"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="57"/>
+      <c r="F41" s="43">
         <f>COUNTIF(F10:F40,"P")</f>
         <v>0</v>
       </c>
-      <c r="G41" s="58">
+      <c r="G41" s="43">
         <f>COUNTIF(G10:G40,"S")</f>
         <v>0</v>
       </c>
-      <c r="H41" s="58">
+      <c r="H41" s="43">
         <f>COUNTIF(H10:H40,"BT")</f>
         <v>0</v>
       </c>
-      <c r="I41" s="58">
+      <c r="I41" s="43">
         <f>COUNTIF(I10:I40,"PM")</f>
         <v>0</v>
       </c>
-      <c r="J41" s="58">
+      <c r="J41" s="43">
         <f>COUNTIF(J10:J40,"V")</f>
         <v>0</v>
       </c>
-      <c r="K41" s="58">
-        <f>COUNTIF(K10:K40,"x")</f>
+      <c r="K41" s="43">
+        <f>COUNTIF(K10:K40,"X")</f>
         <v>0</v>
       </c>
-      <c r="L41" s="85"/>
-      <c r="M41" s="74"/>
-      <c r="N41" s="71"/>
-      <c r="O41" s="59"/>
-      <c r="P41" s="59"/>
+      <c r="L41" s="71"/>
+      <c r="M41" s="56"/>
+      <c r="N41" s="57"/>
+      <c r="O41" s="44"/>
+      <c r="P41" s="44"/>
       <c r="Q41" s="31"/>
       <c r="R41" s="26"/>
     </row>
     <row r="42" spans="1:26" ht="15" customHeight="1">
-      <c r="A42" s="60"/>
-      <c r="B42" s="86"/>
-      <c r="C42" s="76"/>
-      <c r="D42" s="76"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="76"/>
-      <c r="H42" s="76"/>
-      <c r="I42" s="76"/>
-      <c r="J42" s="76"/>
-      <c r="K42" s="76"/>
-      <c r="L42" s="76"/>
-      <c r="M42" s="76"/>
-      <c r="N42" s="76"/>
+      <c r="A42" s="45"/>
+      <c r="B42" s="72"/>
+      <c r="C42" s="59"/>
+      <c r="D42" s="59"/>
+      <c r="E42" s="59"/>
+      <c r="F42" s="59"/>
+      <c r="G42" s="59"/>
+      <c r="H42" s="59"/>
+      <c r="I42" s="59"/>
+      <c r="J42" s="59"/>
+      <c r="K42" s="59"/>
+      <c r="L42" s="59"/>
+      <c r="M42" s="59"/>
+      <c r="N42" s="59"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="15" customHeight="1">
-      <c r="B43" s="89" t="s">
+      <c r="B43" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="C43" s="74"/>
-      <c r="D43" s="74"/>
-      <c r="E43" s="89" t="s">
+      <c r="C43" s="56"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="F43" s="74"/>
-      <c r="G43" s="74"/>
-      <c r="H43" s="71"/>
-      <c r="I43" s="89" t="s">
+      <c r="F43" s="56"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="J43" s="74"/>
-      <c r="K43" s="74"/>
-      <c r="L43" s="74"/>
-      <c r="M43" s="71"/>
-      <c r="N43" s="61"/>
+      <c r="J43" s="56"/>
+      <c r="K43" s="56"/>
+      <c r="L43" s="56"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="46"/>
       <c r="O43" s="1"/>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="15" customHeight="1">
-      <c r="B44" s="90" t="s">
+      <c r="B44" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="C44" s="76"/>
-      <c r="D44" s="77"/>
-      <c r="E44" s="93" t="s">
+      <c r="C44" s="59"/>
+      <c r="D44" s="60"/>
+      <c r="E44" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="F44" s="76"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="77"/>
-      <c r="I44" s="90" t="s">
+      <c r="F44" s="59"/>
+      <c r="G44" s="59"/>
+      <c r="H44" s="60"/>
+      <c r="I44" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="J44" s="76"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="77"/>
+      <c r="J44" s="59"/>
+      <c r="K44" s="59"/>
+      <c r="L44" s="59"/>
+      <c r="M44" s="60"/>
       <c r="N44" s="1"/>
       <c r="Q44" s="1"/>
       <c r="R44" s="1"/>
     </row>
     <row r="45" spans="1:26" ht="15" customHeight="1">
-      <c r="B45" s="91"/>
-      <c r="C45" s="63"/>
-      <c r="D45" s="92"/>
-      <c r="E45" s="91"/>
-      <c r="F45" s="63"/>
-      <c r="G45" s="63"/>
-      <c r="H45" s="92"/>
-      <c r="I45" s="91"/>
-      <c r="J45" s="63"/>
-      <c r="K45" s="63"/>
-      <c r="L45" s="63"/>
-      <c r="M45" s="92"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="61"/>
+      <c r="F45" s="62"/>
+      <c r="G45" s="62"/>
+      <c r="H45" s="63"/>
+      <c r="I45" s="61"/>
+      <c r="J45" s="62"/>
+      <c r="K45" s="62"/>
+      <c r="L45" s="62"/>
+      <c r="M45" s="63"/>
       <c r="N45" s="1"/>
       <c r="Q45" s="1"/>
       <c r="R45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="12" customHeight="1">
-      <c r="B46" s="91"/>
-      <c r="C46" s="63"/>
-      <c r="D46" s="92"/>
-      <c r="E46" s="91"/>
-      <c r="F46" s="63"/>
-      <c r="G46" s="63"/>
-      <c r="H46" s="92"/>
-      <c r="I46" s="91"/>
-      <c r="J46" s="63"/>
-      <c r="K46" s="63"/>
-      <c r="L46" s="63"/>
-      <c r="M46" s="92"/>
+      <c r="B46" s="61"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="61"/>
+      <c r="F46" s="62"/>
+      <c r="G46" s="62"/>
+      <c r="H46" s="63"/>
+      <c r="I46" s="61"/>
+      <c r="J46" s="62"/>
+      <c r="K46" s="62"/>
+      <c r="L46" s="62"/>
+      <c r="M46" s="63"/>
       <c r="N46" s="1"/>
       <c r="Q46" s="1"/>
       <c r="R46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="10.5" customHeight="1">
-      <c r="B47" s="91"/>
-      <c r="C47" s="63"/>
-      <c r="D47" s="92"/>
-      <c r="E47" s="91"/>
-      <c r="F47" s="63"/>
-      <c r="G47" s="63"/>
-      <c r="H47" s="92"/>
-      <c r="I47" s="91"/>
-      <c r="J47" s="63"/>
-      <c r="K47" s="63"/>
-      <c r="L47" s="63"/>
-      <c r="M47" s="92"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="62"/>
+      <c r="G47" s="62"/>
+      <c r="H47" s="63"/>
+      <c r="I47" s="61"/>
+      <c r="J47" s="62"/>
+      <c r="K47" s="62"/>
+      <c r="L47" s="62"/>
+      <c r="M47" s="63"/>
       <c r="N47" s="1"/>
       <c r="Q47" s="1"/>
       <c r="R47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="10.5" customHeight="1">
       <c r="A48" s="15"/>
-      <c r="B48" s="78"/>
-      <c r="C48" s="67"/>
-      <c r="D48" s="79"/>
-      <c r="E48" s="78"/>
-      <c r="F48" s="67"/>
-      <c r="G48" s="67"/>
-      <c r="H48" s="79"/>
-      <c r="I48" s="78"/>
-      <c r="J48" s="67"/>
-      <c r="K48" s="67"/>
-      <c r="L48" s="67"/>
-      <c r="M48" s="79"/>
-      <c r="N48" s="61"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="66"/>
+      <c r="E48" s="64"/>
+      <c r="F48" s="65"/>
+      <c r="G48" s="65"/>
+      <c r="H48" s="66"/>
+      <c r="I48" s="64"/>
+      <c r="J48" s="65"/>
+      <c r="K48" s="65"/>
+      <c r="L48" s="65"/>
+      <c r="M48" s="66"/>
+      <c r="N48" s="46"/>
       <c r="O48" s="15"/>
       <c r="P48" s="15"/>
       <c r="Q48" s="15"/>
@@ -2267,47 +2410,47 @@
       <c r="Z48" s="15"/>
     </row>
     <row r="49" spans="2:18" ht="18" customHeight="1">
-      <c r="B49" s="87" t="s">
+      <c r="B49" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="C49" s="74"/>
-      <c r="D49" s="74"/>
-      <c r="E49" s="87" t="s">
+      <c r="C49" s="56"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="F49" s="74"/>
-      <c r="G49" s="74"/>
-      <c r="H49" s="71"/>
-      <c r="I49" s="87" t="s">
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="57"/>
+      <c r="I49" s="68" t="s">
         <v>32</v>
       </c>
-      <c r="J49" s="74"/>
-      <c r="K49" s="74"/>
-      <c r="L49" s="74"/>
-      <c r="M49" s="71"/>
-      <c r="N49" s="61"/>
+      <c r="J49" s="56"/>
+      <c r="K49" s="56"/>
+      <c r="L49" s="56"/>
+      <c r="M49" s="57"/>
+      <c r="N49" s="46"/>
       <c r="Q49" s="1"/>
       <c r="R49" s="1"/>
     </row>
     <row r="50" spans="2:18" ht="16.5" customHeight="1">
-      <c r="B50" s="88" t="s">
+      <c r="B50" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="C50" s="74"/>
-      <c r="D50" s="74"/>
-      <c r="E50" s="88" t="s">
+      <c r="C50" s="56"/>
+      <c r="D50" s="56"/>
+      <c r="E50" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="F50" s="74"/>
-      <c r="G50" s="74"/>
-      <c r="H50" s="71"/>
-      <c r="I50" s="88" t="s">
+      <c r="F50" s="56"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="57"/>
+      <c r="I50" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="J50" s="74"/>
-      <c r="K50" s="74"/>
-      <c r="L50" s="74"/>
-      <c r="M50" s="71"/>
+      <c r="J50" s="56"/>
+      <c r="K50" s="56"/>
+      <c r="L50" s="56"/>
+      <c r="M50" s="57"/>
       <c r="N50" s="1"/>
       <c r="Q50" s="1"/>
       <c r="R50" s="1"/>
@@ -7084,18 +7227,20 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="P8:P9"/>
-    <mergeCell ref="Q8:Q9"/>
-    <mergeCell ref="R8:R9"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="E43:H43"/>
-    <mergeCell ref="I43:M43"/>
-    <mergeCell ref="B44:D48"/>
-    <mergeCell ref="E44:H48"/>
-    <mergeCell ref="I44:M48"/>
-    <mergeCell ref="E49:H49"/>
-    <mergeCell ref="I49:M49"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:K8"/>
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="E50:H50"/>
     <mergeCell ref="I50:M50"/>
@@ -7105,6 +7250,18 @@
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="L41:N41"/>
     <mergeCell ref="B42:N42"/>
+    <mergeCell ref="B44:D48"/>
+    <mergeCell ref="E44:H48"/>
+    <mergeCell ref="I44:M48"/>
+    <mergeCell ref="E49:H49"/>
+    <mergeCell ref="I49:M49"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="E43:H43"/>
+    <mergeCell ref="I43:M43"/>
     <mergeCell ref="L18:N18"/>
     <mergeCell ref="L19:N19"/>
     <mergeCell ref="L20:N20"/>
@@ -7114,21 +7271,8 @@
     <mergeCell ref="L10:N10"/>
     <mergeCell ref="L11:N11"/>
     <mergeCell ref="L14:N14"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:K8"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:G5"/>
   </mergeCells>
+  <phoneticPr fontId="20" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="landscape"/>
@@ -7137,153 +7281,160 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="B2:O22"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col customWidth="true" max="2" min="1" width="4"/>
-    <col customWidth="true" max="3" min="3" width="6"/>
-    <col customWidth="true" max="5" min="4" width="12"/>
-    <col customWidth="true" max="15" min="6" width="10"/>
+    <col min="1" max="2" width="4" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
+    <col min="6" max="15" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="114" t="s">
+    <row r="2" spans="2:15" ht="18">
+      <c r="B2" s="51" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4">
-      <c r="C4" s="106" t="s">
+    <row r="4" spans="2:15">
+      <c r="C4" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="107" t="s">
+      <c r="E4" s="50" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5">
-      <c r="C5" s="106" t="s">
+    <row r="5" spans="2:15">
+      <c r="C5" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="107" t="s">
+      <c r="E5" s="50" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6">
-      <c r="C6" s="106" t="s">
+    <row r="6" spans="2:15">
+      <c r="C6" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="107" t="s">
+      <c r="E6" s="50" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7">
-      <c r="C7" s="106" t="s">
+    <row r="7" spans="2:15">
+      <c r="C7" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="107" t="s">
+      <c r="E7" s="50" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9">
-      <c r="C9" s="96" t="s">
+    <row r="9" spans="2:15">
+      <c r="C9" s="85" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="96"/>
-      <c r="E9" s="96"/>
-      <c r="F9" s="96"/>
-      <c r="G9" s="96"/>
-      <c r="H9" s="96"/>
-      <c r="I9" s="96"/>
-      <c r="J9" s="96"/>
-      <c r="K9" s="96"/>
-      <c r="L9" s="96"/>
-      <c r="M9" s="96"/>
-      <c r="N9" s="96"/>
-      <c r="O9" s="96"/>
-    </row>
-    <row r="11">
-      <c r="C11" s="96" t="s">
+      <c r="D9" s="85"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="85"/>
+      <c r="G9" s="85"/>
+      <c r="H9" s="85"/>
+      <c r="I9" s="85"/>
+      <c r="J9" s="85"/>
+      <c r="K9" s="85"/>
+      <c r="L9" s="85"/>
+      <c r="M9" s="85"/>
+      <c r="N9" s="85"/>
+      <c r="O9" s="85"/>
+    </row>
+    <row r="11" spans="2:15">
+      <c r="C11" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="96" t="s">
+      <c r="D11" s="85" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="96"/>
-      <c r="F11" s="96" t="s">
+      <c r="E11" s="85"/>
+      <c r="F11" s="85" t="s">
         <v>46</v>
       </c>
-      <c r="G11" s="96"/>
-      <c r="H11" s="96" t="s">
+      <c r="G11" s="85"/>
+      <c r="H11" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="96"/>
-      <c r="J11" s="96"/>
-      <c r="K11" s="96"/>
-      <c r="L11" s="96"/>
-      <c r="M11" s="96"/>
-      <c r="N11" s="96"/>
-      <c r="O11" s="96"/>
-    </row>
-    <row r="12">
-      <c r="C12" s="98" t="s">
+      <c r="I11" s="85"/>
+      <c r="J11" s="85"/>
+      <c r="K11" s="85"/>
+      <c r="L11" s="85"/>
+      <c r="M11" s="85"/>
+      <c r="N11" s="85"/>
+      <c r="O11" s="85"/>
+    </row>
+    <row r="12" spans="2:15">
+      <c r="C12" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="98" t="s">
+      <c r="D12" s="86" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98" t="s">
+      <c r="E12" s="86"/>
+      <c r="F12" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="98"/>
-      <c r="H12" s="99" t="s">
+      <c r="G12" s="86"/>
+      <c r="H12" s="87" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="99"/>
-      <c r="J12" s="99"/>
-      <c r="K12" s="99"/>
-      <c r="L12" s="99"/>
-      <c r="M12" s="99"/>
-      <c r="N12" s="99"/>
-      <c r="O12" s="99"/>
-    </row>
-    <row r="21">
-      <c r="C21" s="104" t="s">
+      <c r="I12" s="87"/>
+      <c r="J12" s="87"/>
+      <c r="K12" s="87"/>
+      <c r="L12" s="87"/>
+      <c r="M12" s="87"/>
+      <c r="N12" s="87"/>
+      <c r="O12" s="87"/>
+    </row>
+    <row r="21" spans="3:14">
+      <c r="C21" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="104"/>
-      <c r="E21" s="104"/>
-      <c r="G21" s="104" t="s">
+      <c r="D21" s="88"/>
+      <c r="E21" s="88"/>
+      <c r="G21" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="104"/>
-      <c r="L21" s="104" t="s">
+      <c r="H21" s="88"/>
+      <c r="I21" s="88"/>
+      <c r="J21" s="88"/>
+      <c r="L21" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="M21" s="104"/>
-      <c r="N21" s="104"/>
-    </row>
-    <row r="22">
-      <c r="C22" s="98" t="s">
+      <c r="M21" s="88"/>
+      <c r="N21" s="88"/>
+    </row>
+    <row r="22" spans="3:14">
+      <c r="C22" s="86" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="98"/>
-      <c r="E22" s="98"/>
-      <c r="G22" s="98" t="s">
+      <c r="D22" s="86"/>
+      <c r="E22" s="86"/>
+      <c r="G22" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="H22" s="98"/>
-      <c r="I22" s="98"/>
-      <c r="J22" s="98"/>
-      <c r="L22" s="98" t="s">
+      <c r="H22" s="86"/>
+      <c r="I22" s="86"/>
+      <c r="J22" s="86"/>
+      <c r="L22" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="M22" s="98"/>
-      <c r="N22" s="98"/>
+      <c r="M22" s="86"/>
+      <c r="N22" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="L22:N22"/>
     <mergeCell ref="C9:O9"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="F11:G11"/>
@@ -7291,13 +7442,8 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="H12:O12"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="L21:N21"/>
-    <mergeCell ref="L22:N22"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>